<commit_message>
Subsanar discrepancias de citas del Capítulo I y verificar notas de Nieva-Fenoll
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFqB7qFXyXBvPWdV8axcUP
</commit_message>
<xml_diff>
--- a/Verificacion_citas_Cap_I.xlsx
+++ b/Verificacion_citas_Cap_I.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen Cap. I" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Verificación Cap. I" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hallazgos Cap. I" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RIS vs. fuentes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Transcripciones textuales" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Cap. I" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificación Cap. I" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallazgos Cap. I" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIS vs. fuentes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transcripciones textuales" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen Cap. I'!$A$1:$B$15</definedName>
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -108,6 +108,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -475,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -522,7 +532,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Notas 1 a 249 (Capítulo I). Solo se verificaron contra las 54 obras del archivo RIS; las obras ajenas al RIS se marcan «Fuera del RIS».</t>
+          <t>Notas 1 a 249 (Capítulo I). Se verificaron contra las 54 obras del RIS y, además, contra el artículo de Nieva-Fenoll (2020) que está en el Drive aunque no figura en el RIS.</t>
         </is>
       </c>
     </row>
@@ -561,7 +571,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9">
@@ -591,7 +601,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -628,7 +638,19 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(1) Ferrer, Prueba sin convicción: el tramo impreso pp. 139-148 no está paginado en las copias descargables; la nota 123 se localizó por contenido (±1 página). (2) Laudan, Truth…, Devis Echandía y SUP-JIN-194/2025 se leyeron mediante el texto que extrae Drive, por exceder el límite de descarga de 10 MB. (3) Las 12 notas de Nieva-Fenoll (2020) no se verificaron por no figurar esa obra en el RIS.</t>
+          <t>(1) Ferrer, Prueba sin convicción: el tramo impreso pp. 139-148 no está paginado en las copias descargables; la nota 123 se localizó por contenido (±1 página). (2) Laudan, Truth…, Devis Echandía y SUP-JIN-194/2025 se leyeron mediante el texto que extrae Drive, por exceder el límite de descarga de 10 MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Correcciones aplicadas</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Las 9 discrepancias se subsanaron en «Tesis_Cap_I-V_citas_corregidas.docx» con control de cambios (autor: Claude, verificación de citas). Se entrega también una versión limpia con los cambios aceptados.</t>
         </is>
       </c>
     </row>
@@ -644,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I250"/>
+  <dimension ref="A1:J250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -656,6 +678,7 @@
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -704,6 +727,11 @@
           <t>Observación / pasaje localizado / corrección sugerida</t>
         </is>
       </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Corrección aplicada en el .docx (control de cambios)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -749,6 +777,7 @@
           <t>p. 358: la Carolina instruye «cómo deben averiguar los indicios y qué partido debe sacarse de ellos»; insuficientes para condena, autorizan el tormento.</t>
         </is>
       </c>
+      <c r="J2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -794,6 +823,7 @@
           <t>pp. 358-359: pena extraordinaria; el Código bávaro (p. 359) formula el sistema más completo y excluye la pena de muerte.</t>
         </is>
       </c>
+      <c r="J3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -839,6 +869,7 @@
           <t>pp. 382-383: equipara el fundamento de la convicción por indicios con el de la confesión y el testimonio (el argumento arranca en p. 381).</t>
         </is>
       </c>
+      <c r="J4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -884,6 +915,7 @@
           <t>p. 360: definición literal del indicio («relación tan íntima... conclusión muy natural»; dos hechos, uno comprobado).</t>
         </is>
       </c>
+      <c r="J5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -929,6 +961,7 @@
           <t>p. 361: «el dedo que señala un objeto»; aislado carece de importancia; gravedad según la certeza de la ley de experiencia.</t>
         </is>
       </c>
+      <c r="J6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -974,6 +1007,7 @@
           <t>pp. 361-362: «nuestras deducciones no descansan nunca sino en una simple posibilidad».</t>
         </is>
       </c>
+      <c r="J7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1019,6 +1053,7 @@
           <t>pp. 365-366: contraindicios; ejemplo del poseedor del objeto robado que prueba haberlo comprado.</t>
         </is>
       </c>
+      <c r="J8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1064,6 +1099,7 @@
           <t>p. 382: la opinión solo queda fija tras «haber ensayado inútilmente todas las explicaciones de disculpa».</t>
         </is>
       </c>
+      <c r="J9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1109,6 +1145,7 @@
           <t>p. 219: «un hecho no es indicio en sí, sino que se convierte en tal cuando una regla de experiencia...»; carácter esencialmente relativo.</t>
         </is>
       </c>
+      <c r="J10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1154,6 +1191,7 @@
           <t>p. 127: con acumulación de indicios «la fuente de presunción no está constituida por cada indicio... sino por su conjunto».</t>
         </is>
       </c>
+      <c r="J11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1199,6 +1237,11 @@
           <t>pp. 571-572 respaldan el Reglamento de 1846 (art. 148) y la LEC de 1855 (art. 317). La frase posterior «su propósito fue liberar al juez de ponderar a los testigos en razón de su número» está en p. 577 (y p. 574), no en 571-572. Sugerencia: ampliar a «pp. 571, 572 y 577» o agregar nota a esa frase.</t>
         </is>
       </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «pp. 571 y 572» → «pp. 571, 572 y 577».</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1244,6 +1287,7 @@
           <t>p. 57: apreciación razonada «sin que esto signifique una libertad arbitraria... sujeto a las reglas de la lógica y de la psicología, con obligación de motivar su conclusión».</t>
         </is>
       </c>
+      <c r="J13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1289,6 +1333,7 @@
           <t>p. 360, nota 1: «Estas espresiones son sinónimas en el fondo; los prácticos y el legislador las emplean indiferentemente».</t>
         </is>
       </c>
+      <c r="J14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1334,6 +1379,7 @@
           <t>pp. 271-272: Mittermaier (sinonimia), Reyes Alvarado (identidad estructural) y tesis mayoritaria de Dei Malatesta y Devis Echandía.</t>
         </is>
       </c>
+      <c r="J15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1379,6 +1425,7 @@
           <t>pp. 55-59: esquema de Toulmin aplicado a la inferencia probatoria (razones, pretensión, garantía: máximas, presunciones, otros enunciados generales).</t>
         </is>
       </c>
+      <c r="J16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1424,6 +1471,7 @@
           <t>pp. 61-62: «Si X, entonces probable Y» / «Si X, entonces probado Y» / «X cuenta como Y».</t>
         </is>
       </c>
+      <c r="J17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1469,6 +1517,7 @@
           <t>p. 62: «las presunciones son enunciados revestidos de autoridad».</t>
         </is>
       </c>
+      <c r="J18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1514,6 +1563,7 @@
           <t>p. 87: presunciones como máximas de experiencia institucionalizadas; si su fundamento es cognoscitivo, deben apoyarse en una inducción sólida.</t>
         </is>
       </c>
+      <c r="J19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1559,6 +1609,7 @@
           <t>pp. 42-43: distinción entre «prueba de indicios» y «prueba por indicios» casi literal.</t>
         </is>
       </c>
+      <c r="J20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1604,6 +1655,7 @@
           <t>p. 220: el indicio como tema de prueba y como fuente de prueba.</t>
         </is>
       </c>
+      <c r="J21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1649,6 +1701,7 @@
           <t>p. 79: «según esta clasificación, todas las pruebas sobre hechos pasados son indirectas (o indiciarias)».</t>
         </is>
       </c>
+      <c r="J22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1694,6 +1747,7 @@
           <t>pp. 93-94: aun el testimonio exige establecer la credibilidad y descartar errores de percepción e interpretación.</t>
         </is>
       </c>
+      <c r="J23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1739,6 +1793,7 @@
           <t>pp. 44-46: nexo de necesariedad lógica (testimonio creído) frente a regularidad empírica de grado variable (indicio).</t>
         </is>
       </c>
+      <c r="J24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1784,6 +1839,7 @@
           <t>pp. 285-286: Dei Malatesta define los indicios necesarios como los que revelan en forma cierta una causa determinada con relación constante de causalidad.</t>
         </is>
       </c>
+      <c r="J25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1829,6 +1885,7 @@
           <t>p. 284: contingentes revelan de modo más o menos probable cierta causa o efecto; exigencia de pluralidad.</t>
         </is>
       </c>
+      <c r="J26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1874,6 +1931,7 @@
           <t>p. 219: las fuentes de presunción no se prestan a análisis ni clasificaciones; la división necessariae/violentae/probabiles/temerariae se refiere al valor probatorio.</t>
         </is>
       </c>
+      <c r="J27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1919,6 +1977,7 @@
           <t>p. 48 (nota): clasificación en indicios equiprobables, de probabilidad prevalente, cualificados y necesarios.</t>
         </is>
       </c>
+      <c r="J28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1964,6 +2023,7 @@
           <t>p. 377: ley austriaca (de 6 de julio de 1833, nota 1) exige en principio tres indicios.</t>
         </is>
       </c>
+      <c r="J29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2009,6 +2069,7 @@
           <t>p. 378: solo cuentan los indicios apoyados en circunstancias distintas e independientes; un mismo hecho cuenta una sola vez.</t>
         </is>
       </c>
+      <c r="J30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2054,6 +2115,7 @@
           <t>p. 280: Cortés Coto recoge a Gorphe: huellas similares repiten la misma presunción; «varios indicios mediatos, que sólo dan un indicio inmediato». Cita de segunda mano correctamente señalada.</t>
         </is>
       </c>
+      <c r="J31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2099,6 +2161,7 @@
           <t>p. 82: «un solo hecho probatorio pero con un alto grado de fiabilidad puede tener un peso mayor que varios hechos probatorios de escasa fiabilidad».</t>
         </is>
       </c>
+      <c r="J32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2144,6 +2207,7 @@
           <t>pp. 83-84: variedad de los hechos probatorios; Cohen: eliminación de hipótesis alternativas.</t>
         </is>
       </c>
+      <c r="J33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2189,6 +2253,7 @@
           <t>p. 76: regla de Hempel sobre cantidad y variedad de los datos favorables.</t>
         </is>
       </c>
+      <c r="J34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2234,6 +2299,7 @@
           <t>pp. 365-366: dos clases de hechos favorables (los que impiden atribuir el crimen y los contraindicios).</t>
         </is>
       </c>
+      <c r="J35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2279,6 +2345,7 @@
           <t>pp. 286-287: Devis Echandía (vía Cortés Coto): indicios y contraindicios no desechables desarticulan el conjunto y rompen su convergencia.</t>
         </is>
       </c>
+      <c r="J36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2324,6 +2391,7 @@
           <t>p. 79: la valoración «no puede ser una operación libre de todo criterio y cargada de subjetividad»; referencias legales «sumamente vagas».</t>
         </is>
       </c>
+      <c r="J37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2369,6 +2437,7 @@
           <t>pp. 64-71: deducción, inducción generalizadora, inducción probabilística y abducción.</t>
         </is>
       </c>
+      <c r="J38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2414,6 +2483,7 @@
           <t>p. 70: abducción; falacia de afirmación del consecuente; fuerza derivada de su potencialidad explicativa.</t>
         </is>
       </c>
+      <c r="J39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2459,6 +2529,7 @@
           <t>pp. 80-91: criterios acerca de los hechos probatorios, de la garantía y de la hipótesis.</t>
         </is>
       </c>
+      <c r="J40" s="7" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2504,6 +2575,7 @@
           <t>p. 80: la ausencia de un criterio no es por sí sola razón para rechazar la inferencia; cumplimiento gradual.</t>
         </is>
       </c>
+      <c r="J41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2549,6 +2621,7 @@
           <t>pp. 92-93: correspondencia entre requisitos jurisprudenciales de la prueba indiciaria y criterios de solidez.</t>
         </is>
       </c>
+      <c r="J42" s="7" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2594,6 +2667,7 @@
           <t>pp. 86-87: máximas de experiencia como conclusiones de inducción ampliativa; Gascón: fundamento cognoscitivo.</t>
         </is>
       </c>
+      <c r="J43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2639,6 +2713,11 @@
           <t>p. 86, nota 35 respalda que no debe haber máximas mejor fundadas que desautoricen el paso. La frase siguiente (desconfiar de reglas construidas ad hoc) está en p. 87, no en p. 86. Sugerencia: «p. 86, nota 35, y p. 87».</t>
         </is>
       </c>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 86, nota 35» → «p. 86, nota 35, y p. 87».</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2684,6 +2763,7 @@
           <t>pp. 49-50: la distinción entre «prueba estricta» e «indicio» sigue a la valoración; después se inaugura la valoración conjunta.</t>
         </is>
       </c>
+      <c r="J45" s="7" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2729,6 +2809,7 @@
           <t>pp. 38-39: metáfora del crucigrama y remisión a Haack, Legalizzare l'epistemologia, pp. 19-21 (nota 52); nexos incompatibles, compatibles o recíprocamente implicados.</t>
         </is>
       </c>
+      <c r="J46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2774,6 +2855,7 @@
           <t>p. 51, nota 85: cita de Haack («a veces lo es»), Legalizzare l'epistemologia, pp. 92-93.</t>
         </is>
       </c>
+      <c r="J47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2819,6 +2901,7 @@
           <t>p. 383: el concurso de indicios conduce «al objeto por diversos caminos: la conclusión que el uno suministra la suministra igualmente el otro».</t>
         </is>
       </c>
+      <c r="J48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2864,6 +2947,7 @@
           <t>p. 324, nota 4: «singularitas testium adminiculativa ó cumulativa»; testimonios sobre hechos diversos que se suceden y completan.</t>
         </is>
       </c>
+      <c r="J49" s="7" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2909,6 +2993,7 @@
           <t>p. 395: presunciones sobre conducta y moralidad «no constituyen verdaderos indicios, sino antes bien adminículos».</t>
         </is>
       </c>
+      <c r="J50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2954,6 +3039,7 @@
           <t>Art. 16, párrs. 1-3, LGSMIME (texto con última reforma DOF 14-11-2025): coincide. Obs.: el párr. 3 enumera también instrumental de actuaciones, confesional, reconocimientos o inspecciones y periciales; la tesis menciona solo cuatro medios (enumeración parcial, no errónea).</t>
         </is>
       </c>
+      <c r="J51" s="7" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2999,6 +3085,7 @@
           <t>Tesis 1a. CCLXXXIII/2013, reg. 2004757: definición, conexión racional, no confundir con «cúmulo de sospechas». Datos de publicación correctos.</t>
         </is>
       </c>
+      <c r="J52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -3044,6 +3131,7 @@
           <t>Voto particular AD 78/2012: reprocha falta de análisis exhaustivo (párrs. 12-17); la mayoría sostuvo que «presunciones abstractas no se contrastaron con otras posibles hipótesis». Obs.: la nota carece de localizador; se sugiere añadir párrafos (p. ej., párrs. 4 y 12-17).</t>
         </is>
       </c>
+      <c r="J53" s="7" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3089,6 +3177,7 @@
           <t>Tesis II.1o.P.1 P (11a.), reg. 2024878: umbral más allá de toda duda razonable; indicios unívocos, concurrentes, convergentes e interrelacionados; STC 175/1985 y 229/1988; Corte IDH.</t>
         </is>
       </c>
+      <c r="J54" s="7" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3134,6 +3223,7 @@
           <t>SUP-JRC-487/2000 (fragmento pp. 470-510): análisis «en dos etapas sucesivas... de manera concatenada, adminiculando entre sí»; testimonios ante notario como indicios. Obs.: el localizador abarca 41 páginas; conviene indicar la página exacta.</t>
         </is>
       </c>
+      <c r="J55" s="7" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3179,6 +3269,7 @@
           <t>Jurisprudencia 38/2002: notas periodísticas solo arrojan indicios; mayor calidad indiciaria si provienen de distintos medios y autores, coinciden y no hay mentís. Supl. 6, 2003, p. 44; precedente SUP-JRC-349/2001 correcto.</t>
         </is>
       </c>
+      <c r="J56" s="7" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -3224,6 +3315,7 @@
           <t>Jurisprudencia 4/2014: carácter imperfecto de las pruebas técnicas; requieren adminicularse. Gaceta año 7, núm. 14, 2014, pp. 23-24.</t>
         </is>
       </c>
+      <c r="J57" s="7" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3269,6 +3361,7 @@
           <t>Tesis XXXI/2004: factores cualitativo y cuantitativo; número cierto o calculable «mediante prueba directa o indirecta, como la indiciaria». Compilación 1997-2005, pp. 725-726.</t>
         </is>
       </c>
+      <c r="J58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3314,6 +3407,7 @@
           <t>Jurisprudencia 9/98: la nulidad solo procede si se acreditan plenamente los extremos de la causal. Supl. 2, 1998, pp. 19-20.</t>
         </is>
       </c>
+      <c r="J59" s="7" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3359,6 +3453,7 @@
           <t>Jurisprudencia 44/2024: las violaciones «deben estar plenamente acreditadas». Gaceta año 17, núm. 29, 2024, pp. 149-151.</t>
         </is>
       </c>
+      <c r="J60" s="7" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3404,6 +3499,11 @@
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párrs. 50-60 están en pp. 10-12 (no 11-13). Contenido conforme: requisitos de indicios e inferencias.</t>
         </is>
       </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «pp. 11-13» → «pp. 10-12».</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3449,6 +3549,7 @@
           <t>SUP-JIN-194/2025, párrs. 90-92: sin pruebas directas de hechos indiciarios, sin pluralidad, sin indicios concomitantes de difusión, autoría o financiamiento.</t>
         </is>
       </c>
+      <c r="J62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3494,6 +3595,7 @@
           <t>p. 37: la «valoración conjunta» parece «ahorrarnos... hasta la más mínima glosa»; baluarte de la valoración más subjetiva e incontrolable.</t>
         </is>
       </c>
+      <c r="J63" s="7" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3539,6 +3641,7 @@
           <t>p. 38: imagen del ramillete frente a la del puré.</t>
         </is>
       </c>
+      <c r="J64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3584,6 +3687,7 @@
           <t>p. 378: cada indicio debe apoyarse en circunstancias distintas e independientes; ejemplo de la pistola.</t>
         </is>
       </c>
+      <c r="J65" s="7" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3629,6 +3733,7 @@
           <t>pp. 75-77: «rendimiento decreciente de las nuevas pruebas» redundantes.</t>
         </is>
       </c>
+      <c r="J66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3674,6 +3779,7 @@
           <t>pp. 86-88: máximas de experiencia probables en sentido inferencial; grado de probabilidad causal.</t>
         </is>
       </c>
+      <c r="J67" s="7" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3719,6 +3825,7 @@
           <t>La tesis II.1o.P.1 P invoca la STC 229/1988 (explicitar el íter mental). Obs.: nota abreviada sin localizador; aceptable por ser tesis de dos páginas.</t>
         </is>
       </c>
+      <c r="J68" s="7" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3764,6 +3871,7 @@
           <t>p. 94, nota 44: fijar criterios por vía jurisprudencial «corre el peligro de instaurar un nuevo sistema de valoración tasada».</t>
         </is>
       </c>
+      <c r="J69" s="7" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3809,6 +3917,7 @@
           <t>p. 377: la ley austriaca exige un número mínimo de indicios.</t>
         </is>
       </c>
+      <c r="J70" s="7" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3854,6 +3963,7 @@
           <t>p. 396: exigir absolutamente indicios anteriores, concomitantes y posteriores obligaría a absolver aun siendo cierta la culpabilidad.</t>
         </is>
       </c>
+      <c r="J71" s="7" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -3899,6 +4009,7 @@
           <t>p. 39: colofón de la valoración conjunta: grado de confirmación según el estándar; lógica del «más o menos».</t>
         </is>
       </c>
+      <c r="J72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3944,6 +4055,7 @@
           <t>pp. 41-49: tres momentos de la actividad probatoria.</t>
         </is>
       </c>
+      <c r="J73" s="7" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3989,6 +4101,7 @@
           <t>p. 48: el resultado de la valoración «no implica por sí solo nada respecto de la decisión»; intermediación de un estándar.</t>
         </is>
       </c>
+      <c r="J74" s="7" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -4034,6 +4147,7 @@
           <t>pp. 47-48: la hipótesis más confirmada no siempre debe darse por probada; ejemplo del estándar penal.</t>
         </is>
       </c>
+      <c r="J75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -4079,6 +4193,7 @@
           <t>p. 51: «compete al legislador fijar el estándar (o el quantum) de prueba exigido».</t>
         </is>
       </c>
+      <c r="J76" s="7" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -4124,6 +4239,7 @@
           <t>p. 18: la necesidad de reglas sobre el grado de probabilidad suficiente «ha sido un tema generalmente olvidado en nuestra cultura jurídica». Obs.: Ferrer dice «nuestra cultura jurídica»; la tesis precisa «continental» (interpretación razonable).</t>
         </is>
       </c>
+      <c r="J77" s="7" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -4169,6 +4285,7 @@
           <t>p. 19: solo con estándares pueden operar las cargas de la prueba y las presunciones.</t>
         </is>
       </c>
+      <c r="J78" s="7" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -4214,6 +4331,7 @@
           <t>Art. 16, párrs. 1-3, LGSMIME: coincide.</t>
         </is>
       </c>
+      <c r="J79" s="7" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -4241,24 +4359,25 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (Estudios de Derecho, 2020) no figura en el RIS (el RIS registra otra obra del autor: La valoración de la prueba, 2010). No se verificó por instrucción de limitarse al RIS.</t>
-        </is>
-      </c>
+          <t>Nieva-Fenoll (PDF en Drive), p. 130: probatio plena (documento público, dos testigos, juramento) y semiplena probatio (documento privado, un testigo); de ella derivaban los indicios.</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -4304,6 +4423,7 @@
           <t>p. 32: «La libre convicción del juez no es persuasión libérrima y sin sujeción a pruebas».</t>
         </is>
       </c>
+      <c r="J81" s="7" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -4349,6 +4469,7 @@
           <t>p. 34: «momento místico» (Andrés Ibáñez) y Ferrajoli: «una de las páginas políticamente más amargas...».</t>
         </is>
       </c>
+      <c r="J82" s="7" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -4394,6 +4515,7 @@
           <t>pp. 141-142: la libre convicción como «principio metodológico (negativo)».</t>
         </is>
       </c>
+      <c r="J83" s="7" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4439,6 +4561,7 @@
           <t>pp. 75-76: STS 10-2-1978 (conciencia, «intención que se presume siempre recta») y STS 2-2-1976; dos consecuencias.</t>
         </is>
       </c>
+      <c r="J84" s="7" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4484,6 +4607,7 @@
           <t>p. 33: Locke y Wilkins, «moral certainty» frente a certeza matemática; juez Shaw (1850).</t>
         </is>
       </c>
+      <c r="J85" s="7" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4529,6 +4653,7 @@
           <t>p. 34: In re Winship dio «constitutional imprimatur» al BARD; Commonwealth v. Webster, 59 Mass. 295 (1850).</t>
         </is>
       </c>
+      <c r="J86" s="7" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -4556,24 +4681,25 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 131, nota 56: «Así se hizo hacia 1780 en el Old Bailey de Londres, como relata Whitman (2005)»; el BARD como «simple instrucción para jurados».</t>
+        </is>
+      </c>
+      <c r="J87" s="7" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4601,24 +4727,25 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 132: preponderance of evidence / balance of probabilities, clear and convincing evidence y BARD; recuerdan a la probatio plena y semiplena.</t>
+        </is>
+      </c>
+      <c r="J88" s="7" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -4646,24 +4773,25 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H89" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 133: Beweismaß; probabilidad preponderante, BARD y Glaubhaftmachung (estándar mínimo para medidas cautelares); «ninguna familia jurídica ha sido ajena».</t>
+        </is>
+      </c>
+      <c r="J89" s="7" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -4709,6 +4837,7 @@
           <t>p. 172: «tres factores cruciales empujan a los sistemas probatorios anglosajones hacia la convergencia... en la subjetividad».</t>
         </is>
       </c>
+      <c r="J90" s="7" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -4754,6 +4883,7 @@
           <t>p. 173: la incorporación del BARD sin definición deja todo «remitido a la subjetividad del juzgador».</t>
         </is>
       </c>
+      <c r="J91" s="7" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -4799,6 +4929,7 @@
           <t>p. 30: los legisladores vinculan el resultado probatorio «al convencimiento del juzgador».</t>
         </is>
       </c>
+      <c r="J92" s="7" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -4844,6 +4975,7 @@
           <t>pp. 20-21: art. 316 CNPP («indicios razonables») y art. 530 del Codice di procedura penale.</t>
         </is>
       </c>
+      <c r="J93" s="7" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -4889,6 +5021,7 @@
           <t>Vázquez (ed.), p. 24: tres momentos «lógicamente distintos y sucesivos, aunque... pueden presentarse entrelazados».</t>
         </is>
       </c>
+      <c r="J94" s="7" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -4934,6 +5067,7 @@
           <t>Vázquez (ed.), pp. 24-26: reglas jurídicas en el primer y tercer momentos; racionalidad general en el segundo.</t>
         </is>
       </c>
+      <c r="J95" s="7" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -4979,6 +5113,7 @@
           <t>p. 23: valoración individual (fiabilidad) y conjunta (grado de corroboración de cada hipótesis).</t>
         </is>
       </c>
+      <c r="J96" s="7" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -5024,6 +5159,7 @@
           <t>Vázquez (ed.), p. 26: resultado «siempre contextual»; libre valoración libre solo frente a normas que predeterminen el resultado.</t>
         </is>
       </c>
+      <c r="J97" s="7" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -5069,6 +5205,7 @@
           <t>p. 23: «las pruebas subdeterminan la decisión probatoria»; tres tipos de reglas de decisión.</t>
         </is>
       </c>
+      <c r="J98" s="7" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -5114,6 +5251,7 @@
           <t>p. 48: el resultado de la valoración no implica por sí solo nada respecto de la decisión.</t>
         </is>
       </c>
+      <c r="J99" s="7" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -5159,6 +5297,7 @@
           <t>p. 23, nota 15: Tuzet (2020: 94) muestra la confusión, en especial del TEDH.</t>
         </is>
       </c>
+      <c r="J100" s="7" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -5204,6 +5343,7 @@
           <t>Tesis II.1o.P.1 P: el ejercicio inferencial es válido pero su resultado debe satisfacer el umbral más allá de toda duda razonable.</t>
         </is>
       </c>
+      <c r="J101" s="7" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -5249,6 +5389,7 @@
           <t>Vázquez, «A modo de presentación», p. 14: decisión de política pública; la epistemología dice «el cómo pero no el cuánto».</t>
         </is>
       </c>
+      <c r="J102" s="7" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -5294,6 +5435,7 @@
           <t>pp. 23-24 (y nota): el estándar farmacológico es más elevado que el de la historia por el coste del error.</t>
         </is>
       </c>
+      <c r="J103" s="7" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -5339,6 +5481,7 @@
           <t>p. 149: «el debido proceso exige que el legislador determine para cada tipo de casos el umbral... pero no requiere alguno en particular».</t>
         </is>
       </c>
+      <c r="J104" s="7" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -5384,6 +5527,7 @@
           <t>p. 115: falso positivo / falso negativo; el error material puede darse con razonamiento correcto.</t>
         </is>
       </c>
+      <c r="J105" s="7" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -5429,6 +5573,7 @@
           <t>pp. 29-30: «error distribution doctrine»; estándar, presunción de inocencia, beneficio de la duda y carga de la prueba no están diseñados para reducir errores sino para distribuirlos.</t>
         </is>
       </c>
+      <c r="J106" s="7" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -5474,6 +5619,7 @@
           <t>pp. 116-122: elevar el umbral (0,7 frente a 0,5) disminuye condenas falsas pero aumenta más las absoluciones falsas.</t>
         </is>
       </c>
+      <c r="J107" s="7" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -5519,6 +5665,7 @@
           <t>pp. 121-122: dos estrategias: reducción de errores (acervo probatorio) y distribución del riesgo (preferencias morales o políticas).</t>
         </is>
       </c>
+      <c r="J108" s="7" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -5564,6 +5711,7 @@
           <t>Laudan en Vázquez (ed.), pp. 121-122: ratio de Blackstone (Maimónides, Franklin, Hale, Voltaire).</t>
         </is>
       </c>
+      <c r="J109" s="7" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -5609,6 +5757,7 @@
           <t>Vázquez (ed.), pp. 122-123: las estimaciones «difieren en un factor de 500»; ninguna fue debatida ni defendida.</t>
         </is>
       </c>
+      <c r="J110" s="7" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -5654,6 +5803,7 @@
           <t>p. 109: tres funciones de los estándares.</t>
         </is>
       </c>
+      <c r="J111" s="7" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -5699,6 +5849,7 @@
           <t>p. 115: las dos primeras funciones se cumplen por su mera existencia; la tercera depende del umbral; crítica a la doctrina mayoritaria.</t>
         </is>
       </c>
+      <c r="J112" s="7" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -5744,6 +5895,7 @@
           <t>pp. 109-110: función heurística y justificativa (Gascón Abellán).</t>
         </is>
       </c>
+      <c r="J113" s="7" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -5789,6 +5941,7 @@
           <t>pp. 112-114: la indeterminación del umbral «vacía de contenido el propio derecho al recurso».</t>
         </is>
       </c>
+      <c r="J114" s="7" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -5816,24 +5969,25 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H115" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 118 (resumen): carga y estándares provienen del sistema de valoración legal; «simples remedos» imposibles de objetivar.</t>
+        </is>
+      </c>
+      <c r="J115" s="7" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -5861,24 +6015,25 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H116" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 133: la probabilidad preponderante «no es ninguna herramienta que ayude al juez, sino... una simple descripción de su labor cotidiana».</t>
+        </is>
+      </c>
+      <c r="J116" s="7" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -5906,24 +6061,25 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H117" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 134: en el sistema estadounidense nadie motiva el cumplimiento de los estándares (jurado).</t>
+        </is>
+      </c>
+      <c r="J117" s="7" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -5969,6 +6125,7 @@
           <t>p. 26: «el origen histórico de una institución nada dice acerca de su necesidad conceptual».</t>
         </is>
       </c>
+      <c r="J118" s="7" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -6014,6 +6171,7 @@
           <t>p. 110: prueba legal y estándares son incompatibles; el estándar presupone el razonamiento probatorio.</t>
         </is>
       </c>
+      <c r="J119" s="7" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -6059,6 +6217,7 @@
           <t>Vázquez, «A modo de presentación», p. 14: no es regreso a la prueba tasada; los estándares operan sobre el conjunto.</t>
         </is>
       </c>
+      <c r="J120" s="7" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -6104,6 +6263,7 @@
           <t>pp. 110-111: analogía de Anderson, Schum y Twining sobre la nota mínima de aprobación.</t>
         </is>
       </c>
+      <c r="J121" s="7" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -6149,6 +6309,7 @@
           <t>Art. 15, párr. 2, LGSMIME: «El que afirma está obligado a probar. También lo está el que niega...».</t>
         </is>
       </c>
+      <c r="J122" s="7" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -6194,6 +6355,7 @@
           <t>p. 19: la carga determina quién pierde si no hay prueba suficiente, «pero para aplicarlas es necesario conocer cuándo hay prueba suficiente».</t>
         </is>
       </c>
+      <c r="J123" s="7" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -6239,6 +6401,7 @@
           <t>Nota 95: «el riesgo de error nunca es del todo simétrico, por efecto de la carga de la prueba» (Bell, 1987). Obs.: el tramo impreso pp. 139-148 no está paginado en las copias disponibles; el texto de la nota 95 se localizó pero la página 142 solo pudo confirmarse por aproximación (±1).</t>
         </is>
       </c>
+      <c r="J124" s="7" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -6284,6 +6447,7 @@
           <t>p. 30: la asignación de la carga de la prueba al fiscal figura entre los principios de distribución del error.</t>
         </is>
       </c>
+      <c r="J125" s="7" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -6311,24 +6475,25 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H126" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 128: la carga objetiva se identifica con la valoración; el concepto «se convierte en redundante».</t>
+        </is>
+      </c>
+      <c r="J126" s="7" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -6374,6 +6539,11 @@
           <t>p. 48 existe y expone la regla de la presunción de determinancia (&lt;5 %). Pero la Sala NO la aplicó: la diferencia era de 45,922 votos (11.11 %), por lo que sostuvo que la carga correspondía a quien pretendía la nulidad (pp. 48-49). La tesis afirma que «aplicó la presunción». Sugerencia: «la Sala Superior invocó la presunción de determinancia (&lt;5 %) y, al superar la diferencia ese umbral (11.11 %), atribuyó la carga a quien pedía la nulidad (pp. 48-49)». El argumento de la tesis (confusión carga/estándar) se mantiene.</t>
         </is>
       </c>
+      <c r="J127" s="7" t="inlineStr">
+        <is>
+          <t>Texto: «aplicó» → «invocó» y se añadió: «Como la diferencia entre el primero y el segundo lugar era de 11.11 por ciento, atribuyó la carga de acreditar la determinancia a quien pretendía la nulidad.» Nota: «p. 48» → «pp. 48 y 49».</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -6419,6 +6589,7 @@
           <t>p. 46: «el estándar probatorio para analizar la determinancia debe ser mínimo... de tal manera que no implique una carga excesiva o imposible».</t>
         </is>
       </c>
+      <c r="J128" s="7" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -6464,6 +6635,7 @@
           <t>p. 41: «no hay forma de conocer su trascendencia... debe regir la presunción de validez».</t>
         </is>
       </c>
+      <c r="J129" s="7" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -6509,6 +6681,7 @@
           <t>Voto razonado, p. 75: la carga de acreditar la trascendencia fija «un estándar probatorio muy alto, prácticamente imposible de alcanzar».</t>
         </is>
       </c>
+      <c r="J130" s="7" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
@@ -6554,6 +6727,7 @@
           <t>CNPP (reforma DOF 28-11-2025), art. 259 («de manera libre y lógica») y art. 265 («apreciación conjunta, integral y armónica»).</t>
         </is>
       </c>
+      <c r="J131" s="7" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
@@ -6599,6 +6773,7 @@
           <t>p. 79: referencias legales a lógica, sana crítica y experiencia «sumamente vagas».</t>
         </is>
       </c>
+      <c r="J132" s="7" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
@@ -6644,6 +6819,7 @@
           <t>p. 110: los estándares presuponen el razonamiento probatorio; «solo después de esa labor, procederá la aplicación del estándar».</t>
         </is>
       </c>
+      <c r="J133" s="7" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
@@ -6689,6 +6865,7 @@
           <t>pp. 24-25: argumento de Bayón y réplica de Ferrer.</t>
         </is>
       </c>
+      <c r="J134" s="7" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
@@ -6734,6 +6911,7 @@
           <t>pp. 176-179: tres razones, «cada una de ellas suficientes por sí solas», contra vincular prueba y creencia del juzgador.</t>
         </is>
       </c>
+      <c r="J135" s="7" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -6779,6 +6957,7 @@
           <t>p. 192: no tiene sentido exigir justificación del hecho mental de creer; la concepción subjetivista «nunca haya requerido la motivación».</t>
         </is>
       </c>
+      <c r="J136" s="7" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
@@ -6824,6 +7003,7 @@
           <t>p. 193: estándares con «criterios intersubjetivamente controlables» sobre la capacidad justificativa de las pruebas.</t>
         </is>
       </c>
+      <c r="J137" s="7" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
@@ -6869,6 +7049,7 @@
           <t>CPEUM (últimas reformas DOF 02-06-2026), art. 16, párr. primero: acto de molestia que «funde y motive la causa legal del procedimiento».</t>
         </is>
       </c>
+      <c r="J138" s="7" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
@@ -6914,6 +7095,7 @@
           <t>p. 51: glosas del BARD definidas por «the target mental state of the juror».</t>
         </is>
       </c>
+      <c r="J139" s="7" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
@@ -6959,6 +7141,7 @@
           <t>p. 52: ejemplo del matemático; «the robustness of its proof, not the confidence of its discoverer».</t>
         </is>
       </c>
+      <c r="J140" s="7" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
@@ -7004,6 +7187,7 @@
           <t>p. 53: criterios subjetivos frente a conexiones lógicas entre prueba y veredicto.</t>
         </is>
       </c>
+      <c r="J141" s="7" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
@@ -7049,6 +7233,7 @@
           <t>p. 80: «Outside the law, rational confidence in a conjecture follows on its proof... Inside the law, such confidence precedes, certifies, and even constitutes the “proof”».</t>
         </is>
       </c>
+      <c r="J142" s="7" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -7094,6 +7279,7 @@
           <t>p. 81: «not a SoP but a pretext... for a conviction or for an acquittal».</t>
         </is>
       </c>
+      <c r="J143" s="7" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
@@ -7139,6 +7325,7 @@
           <t>p. 82: fórmula a) sobre prueba inculpatoria difícil de explicar si fuera inocente.</t>
         </is>
       </c>
+      <c r="J144" s="7" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
@@ -7184,6 +7371,7 @@
           <t>pp. 76-78: epistemología subyacente a la íntima convicción e «implicaciones tan asombrosas».</t>
         </is>
       </c>
+      <c r="J145" s="7" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
@@ -7229,6 +7417,7 @@
           <t>p. 177, nota 18: Taruffo (2009c: 104): «la intensidad y la profundidad del convencimiento no garantizan de ningún modo la verdad de su objeto».</t>
         </is>
       </c>
+      <c r="J146" s="7" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
@@ -7274,6 +7463,7 @@
           <t>CPEUM art. 20, A, VIII («El juez sólo condenará cuando exista convicción de la culpabilidad del procesado») y B, I (presunción de inocencia).</t>
         </is>
       </c>
+      <c r="J147" s="7" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
@@ -7319,6 +7509,7 @@
           <t>CNPP arts. 359 y 402: convicción de la culpabilidad «más allá de toda duda razonable».</t>
         </is>
       </c>
+      <c r="J148" s="7" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
@@ -7364,6 +7555,7 @@
           <t>p. 30: incluye el art. 20.A.VIII CPEUM y el art. 402 CNPP entre los ejemplos de vinculación del resultado probatorio a la convicción.</t>
         </is>
       </c>
+      <c r="J149" s="7" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
@@ -7391,24 +7583,25 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H150" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 131, nota 54: cita el art. 359 del CNPP (y el art. 340 del CPP chileno).</t>
+        </is>
+      </c>
+      <c r="J150" s="7" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
@@ -7454,6 +7647,7 @@
           <t>p. 97: la SCJN sostiene que la duda razonable «opera como estándar objetivo de valoración probatoria»; nota 17: P./J. 8/2023 (11a.), reg. 2027822.</t>
         </is>
       </c>
+      <c r="J151" s="7" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
@@ -7499,6 +7693,7 @@
           <t>p. 98: «aquella labor intelectual, netamente subjetiva, del impartidor de justicia».</t>
         </is>
       </c>
+      <c r="J152" s="7" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n">
@@ -7544,6 +7739,11 @@
           <t>La característica «2. Naturaleza objetiva: No debe basarse en percepciones personales del juzgador» está en p. 98, no en p. 99 (p. 99 contiene las características 3 a 5). Sugerencia: «p. 98» o «pp. 98 y 99».</t>
         </is>
       </c>
+      <c r="J153" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 99» → «p. 98».</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
@@ -7589,6 +7789,7 @@
           <t>CPEUM art. 41, base VI: violaciones «deberán acreditarse de manera objetiva y material»; presunción de determinancia &lt;5 %.</t>
         </is>
       </c>
+      <c r="J154" s="7" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
@@ -7634,6 +7835,7 @@
           <t>LGSMIME arts. 75.1.k («plenamente acreditadas»), 77 Ter.2, 78.1 y 78 bis.2: coinciden.</t>
         </is>
       </c>
+      <c r="J155" s="7" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -7679,6 +7881,7 @@
           <t>Jurisprudencia 44/2024: violaciones «plenamente acreditadas».</t>
         </is>
       </c>
+      <c r="J156" s="7" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
@@ -7724,6 +7927,11 @@
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 39 (estándar flexible; imposible demostrar de manera directa) está en p. 7, no en p. 8.</t>
         </is>
       </c>
+      <c r="J157" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 8» → «p. 7».</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
@@ -7769,6 +7977,11 @@
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 45 («consecuencia más extrema y lesiva»; plena acreditación) está en p. 8, no en p. 9.</t>
         </is>
       </c>
+      <c r="J158" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 9» → «p. 8».</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n">
@@ -7814,6 +8027,11 @@
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 50 («escuela de libre investigación o libre convencimiento»; «formulación racional y controlable») está en p. 10, no en p. 11.</t>
         </is>
       </c>
+      <c r="J159" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 11» → «p. 10».</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
@@ -7859,6 +8077,7 @@
           <t>SUP-REC-1388/2018, p. 46: estándar «mínimo» para la determinancia en casos de violencia política.</t>
         </is>
       </c>
+      <c r="J160" s="7" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n">
@@ -7904,6 +8123,7 @@
           <t>p. 28: el particularismo «no puede ser epistémico... sino político-moral».</t>
         </is>
       </c>
+      <c r="J161" s="7" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n">
@@ -7949,6 +8169,7 @@
           <t>p. 28: Nance: sin estándares predeterminados «decae el estado de derecho mismo».</t>
         </is>
       </c>
+      <c r="J162" s="7" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n">
@@ -7994,6 +8215,7 @@
           <t>p. 114: los estándares permiten argumentar errores en la identificación o aplicación del estándar.</t>
         </is>
       </c>
+      <c r="J163" s="7" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n">
@@ -8039,6 +8261,7 @@
           <t>p. 192, nota 66: «un tribunal superior lo máximo que podrá decir es que su creencia es otra y manda más».</t>
         </is>
       </c>
+      <c r="J164" s="7" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
@@ -8084,6 +8307,7 @@
           <t>Jurisprudencia 9/98: principio de conservación de los actos públicos válidamente celebrados.</t>
         </is>
       </c>
+      <c r="J165" s="7" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
@@ -8129,6 +8353,7 @@
           <t>p. 114: presunciones iuris tantum presuponen el umbral de suficiencia a partir del cual se derrotan.</t>
         </is>
       </c>
+      <c r="J166" s="7" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n">
@@ -8174,6 +8399,7 @@
           <t>p. 29: tres requisitos metodológicos más un cuarto.</t>
         </is>
       </c>
+      <c r="J167" s="7" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n">
@@ -8219,6 +8445,7 @@
           <t>pp. 29-30: el primer requisito excluye criterios que remitan a estados mentales del juzgador.</t>
         </is>
       </c>
+      <c r="J168" s="7" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
@@ -8260,6 +8487,7 @@
           <t>p. 29: requisitos metodológicos.</t>
         </is>
       </c>
+      <c r="J169" s="7" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
@@ -8305,6 +8533,7 @@
           <t>p. 29: tres requisitos y un cuarto sobre la relación entre estándares de un mismo proceso.</t>
         </is>
       </c>
+      <c r="J170" s="7" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
@@ -8350,6 +8579,7 @@
           <t>p. 29, nota 1: «Doy por supuesto... que estamos ante una regla general y abstracta».</t>
         </is>
       </c>
+      <c r="J171" s="7" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n">
@@ -8395,6 +8625,7 @@
           <t>p. 29: se excluye toda formulación que remita a estados mentales o psicológicos del juzgador.</t>
         </is>
       </c>
+      <c r="J172" s="7" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
@@ -8440,6 +8671,7 @@
           <t>pp. 29-30: ejemplos legislativos (íntima convicción, convicción del tribunal), incluidos art. 20.A.VIII CPEUM y art. 402 CNPP.</t>
         </is>
       </c>
+      <c r="J173" s="7" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
@@ -8485,6 +8717,7 @@
           <t>CPEUM art. 20.A.VIII: «El juez sólo condenará cuando exista convicción de la culpabilidad del procesado».</t>
         </is>
       </c>
+      <c r="J174" s="7" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
@@ -8530,6 +8763,7 @@
           <t>CNPP art. 402: convicción del tribunal «más allá de toda duda razonable».</t>
         </is>
       </c>
+      <c r="J175" s="7" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
@@ -8575,6 +8809,7 @@
           <t>p. 32: del convencimiento psicológico respecto de «p» no se infiere nada acerca de su verdad ni de su corroboración.</t>
         </is>
       </c>
+      <c r="J176" s="7" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
@@ -8620,6 +8855,7 @@
           <t>p. 33: siguiendo a Laudan, lo determinante es si «sería racional tenerla» a la luz de las pruebas.</t>
         </is>
       </c>
+      <c r="J177" s="7" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
@@ -8665,6 +8901,7 @@
           <t>pp. 51-53: crítica a las glosas subjetivas del BARD y exigencia de conexión lógica entre prueba y veredicto.</t>
         </is>
       </c>
+      <c r="J178" s="7" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
@@ -8710,6 +8947,7 @@
           <t>p. 31, nota 4: ADR 3457/2013 y tesis 1a. CCXVIII/2015, reg. 2009462.</t>
         </is>
       </c>
+      <c r="J179" s="7" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
@@ -8755,6 +8993,7 @@
           <t>Art. 16, párr. 3, LGSMIME: «generen convicción sobre la veracidad de los hechos afirmados».</t>
         </is>
       </c>
+      <c r="J180" s="7" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
@@ -8800,6 +9039,7 @@
           <t>pp. 33-34: no satisfacen el requisito las remisiones a la inducción o a las leyes de la lógica o la ciencia; exigencias distintas según el estadio.</t>
         </is>
       </c>
+      <c r="J181" s="7" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
@@ -8845,6 +9085,7 @@
           <t>p. 34: no basta decir que la decisión debe estar inductivamente justificada; es necesario determinar el umbral.</t>
         </is>
       </c>
+      <c r="J182" s="7" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n">
@@ -8890,6 +9131,7 @@
           <t>p. 35: solo valores numéricos darían precisión total, lo que infringe el tercer requisito; residuo de vaguedad ineliminable.</t>
         </is>
       </c>
+      <c r="J183" s="7" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
@@ -8935,6 +9177,7 @@
           <t>p. 35, nota 17: Khawaja v. Secretary of State [1984] AC 74, HL, citado por Roberts y Zuckerman: «es, en gran medida, una cuestión de palabras».</t>
         </is>
       </c>
+      <c r="J184" s="7" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n">
@@ -8980,6 +9223,7 @@
           <t>p. 34 (nota): Posner (2001: 367): jueces federales sitúan el BARD entre el 75 y el 95 por 100.</t>
         </is>
       </c>
+      <c r="J185" s="7" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
@@ -9025,6 +9269,7 @@
           <t>p. 35: con Laudan, la fórmula «no merece el nombre de estándar de prueba».</t>
         </is>
       </c>
+      <c r="J186" s="7" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n">
@@ -9070,6 +9315,7 @@
           <t>pp. 35-43: objeciones de Bayón, Dei Vecchi y González Lagier sobre la gradualidad de los criterios.</t>
         </is>
       </c>
+      <c r="J187" s="7" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n">
@@ -9115,6 +9361,7 @@
           <t>pp. 38-39: González Lagier y la comparación ordinal de hipótesis según criterios epistémicos.</t>
         </is>
       </c>
+      <c r="J188" s="7" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n">
@@ -9160,6 +9407,7 @@
           <t>p. 40: resultados probatorios mínimos (refutar todas las hipótesis compatibles con la inocencia, etc.).</t>
         </is>
       </c>
+      <c r="J189" s="7" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n">
@@ -9205,6 +9453,7 @@
           <t>pp. 40-43: regreso al infinito, problema general de la inducción y división del trabajo cognitivo.</t>
         </is>
       </c>
+      <c r="J190" s="7" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n">
@@ -9250,6 +9499,7 @@
           <t>p. 43: González Lagier admite que algunos estándares son «mínimamente informativos».</t>
         </is>
       </c>
+      <c r="J191" s="7" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n">
@@ -9295,6 +9545,7 @@
           <t>p. 44: sin razones que apelen a los resultados exigidos por el estándar «no es posible justificar las decisiones».</t>
         </is>
       </c>
+      <c r="J192" s="7" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n">
@@ -9340,6 +9591,7 @@
           <t>pp. 44-53: particularismo frente a universalismo; razón subyacente sobre el daño y el riesgo de error.</t>
         </is>
       </c>
+      <c r="J193" s="7" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
@@ -9385,6 +9637,7 @@
           <t>p. 53: «cuanto mayor sea el daño que la decisión probatoria pueda causar, menor debe ser el riesgo del error...».</t>
         </is>
       </c>
+      <c r="J194" s="7" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n">
@@ -9430,6 +9683,7 @@
           <t>p. 65: la ausencia de estándares legalmente previstos vulnera el debido proceso y el derecho a la prueba.</t>
         </is>
       </c>
+      <c r="J195" s="7" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n">
@@ -9475,6 +9729,7 @@
           <t>p. 65, nota 113: Santosky v. Kramer, 455 U.S., p. 757 (1982).</t>
         </is>
       </c>
+      <c r="J196" s="7" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
@@ -9520,6 +9775,7 @@
           <t>p. 29: tercer requisito (criterios cualitativos, probabilidad no matemática).</t>
         </is>
       </c>
+      <c r="J197" s="7" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
@@ -9565,6 +9821,7 @@
           <t>p. 65 (y nota 116): vinculación entre los criterios del estándar y el sistema de valoración.</t>
         </is>
       </c>
+      <c r="J198" s="7" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
@@ -9610,6 +9867,7 @@
           <t>pp. 71-73: casos de los autobuses azules (80 %) y del colado (Cohen: 499 entradas, mil asistentes).</t>
         </is>
       </c>
+      <c r="J199" s="7" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n">
@@ -9655,6 +9913,7 @@
           <t>p. 73: «no le interesa el acierto por casualidad»; decisión no justificada sin corroboración suficiente.</t>
         </is>
       </c>
+      <c r="J200" s="7" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
@@ -9700,6 +9959,7 @@
           <t>pp. 74-75: problema de la clase de referencia.</t>
         </is>
       </c>
+      <c r="J201" s="7" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
@@ -9745,6 +10005,7 @@
           <t>Haack en Vázquez (ed.), p. 66: estándares como grados de aval, no identificables con probabilidades matemáticas; «probabilismo jurídico».</t>
         </is>
       </c>
+      <c r="J202" s="7" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
@@ -9790,6 +10051,7 @@
           <t>Haack, p. 78: usos epistemológicos y estadísticos de «probable» «relevantemente diferentes».</t>
         </is>
       </c>
+      <c r="J203" s="7" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
@@ -9835,6 +10097,7 @@
           <t>pp. 89-90: probabilidad inductiva baconiana; no rigen complementariedad ni multiplicación.</t>
         </is>
       </c>
+      <c r="J204" s="7" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
@@ -9880,6 +10143,7 @@
           <t>p. 91: conjunción igual a la hipótesis de menor apoyo; ejemplo de la estafa.</t>
         </is>
       </c>
+      <c r="J205" s="7" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
@@ -9925,6 +10189,7 @@
           <t>Haack, pp. 81-82: tres elementos con 0,51 «sólo tendrían una probabilidad en conjunto de 0,13».</t>
         </is>
       </c>
+      <c r="J206" s="7" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n">
@@ -9970,6 +10235,11 @@
           <t>Haack: la metáfora del crucigrama está en p. 78 ✓, pero la afirmación de que una agregación puede avalar la conclusión en grado mayor que sus componentes está en p. 82 (no en p. 81). Sugerencia: «pp. 78 y 82».</t>
         </is>
       </c>
+      <c r="J207" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «pp. 78 y 81» → «pp. 78 y 82».</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
@@ -10015,6 +10285,7 @@
           <t>Haack, p. 82: «la combinación de pruebas siempre es más fuerte... sino que a veces lo es».</t>
         </is>
       </c>
+      <c r="J208" s="7" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
@@ -10060,6 +10331,7 @@
           <t>pp. 92-99: inducción eliminativa; Semmelweis; esquema H y SA y CI → P.</t>
         </is>
       </c>
+      <c r="J209" s="7" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
@@ -10105,6 +10377,7 @@
           <t>p. 100: más hipótesis rivales eliminadas, mayor corroboración; probabilidad inductiva baconiana.</t>
         </is>
       </c>
+      <c r="J210" s="7" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
@@ -10150,6 +10423,7 @@
           <t>Igartua, p. 48, nota 77: escala de indicios equiprobables a necesarios.</t>
         </is>
       </c>
+      <c r="J211" s="7" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n">
@@ -10195,6 +10469,7 @@
           <t>pp. 100-102: cuarto requisito; tendencia ascendente de los estándares en un mismo proceso.</t>
         </is>
       </c>
+      <c r="J212" s="7" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n">
@@ -10240,6 +10515,7 @@
           <t>p. 102: sobreseimiento &lt; apertura de juicio oral &lt; decisión final.</t>
         </is>
       </c>
+      <c r="J213" s="7" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n">
@@ -10285,6 +10561,7 @@
           <t>p. 103: no exigible un estándar tan exigente en estadios iniciales; ordenar en progresiva disminución.</t>
         </is>
       </c>
+      <c r="J214" s="7" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n">
@@ -10330,6 +10607,7 @@
           <t>p. 102, nota 233: posible sesgo favorable a reiterar el mismo resultado probatorio.</t>
         </is>
       </c>
+      <c r="J215" s="7" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n">
@@ -10375,6 +10653,7 @@
           <t>Art. 16, párr. 4, LGSMIME: pruebas supervenientes antes del cierre de la instrucción.</t>
         </is>
       </c>
+      <c r="J216" s="7" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n">
@@ -10420,6 +10699,7 @@
           <t>pp. 103-105: crítica a Ferrua (vinculación conceptual entre «prueba» y BARD).</t>
         </is>
       </c>
+      <c r="J217" s="7" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n">
@@ -10465,6 +10745,7 @@
           <t>p. 115: las dos primeras funciones no dependen del nivel de exigencia; la tercera sí.</t>
         </is>
       </c>
+      <c r="J218" s="7" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n">
@@ -10510,6 +10791,7 @@
           <t>pp. 153-154: ubicar el umbral aumenta o disminuye el riesgo de decisión errónea; «Esta es la decisión política...».</t>
         </is>
       </c>
+      <c r="J219" s="7" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n">
@@ -10555,6 +10837,7 @@
           <t>Laudan en Vázquez (ed.), pp. 121-123: ratio de Blackstone y cuánto peor es la falsa condena.</t>
         </is>
       </c>
+      <c r="J220" s="7" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n">
@@ -10600,6 +10883,7 @@
           <t>p. 115, nota 15: la doctrina mayoritaria focaliza la función distributiva; ejemplo de Laudan.</t>
         </is>
       </c>
+      <c r="J221" s="7" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n">
@@ -10645,6 +10929,7 @@
           <t>p. 138: mejorar el peso de los acervos y la formación en razonamiento probatorio es «la única política» que reduce ambos errores.</t>
         </is>
       </c>
+      <c r="J222" s="7" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n">
@@ -10690,6 +10975,7 @@
           <t>p. 150: principios de Dworkin (igualdad y respeto de compromisos asumidos); reglas generales, prohibición de retroactividad.</t>
         </is>
       </c>
+      <c r="J223" s="7" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n">
@@ -10735,6 +11021,7 @@
           <t>p. 151: «verdadera incertidumbre» en sentido de Knight.</t>
         </is>
       </c>
+      <c r="J224" s="7" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n">
@@ -10780,6 +11067,7 @@
           <t>p. 152: no hay mecanismo para cuantificar globalmente los errores ni desagregarlos.</t>
         </is>
       </c>
+      <c r="J225" s="7" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n">
@@ -10825,6 +11113,7 @@
           <t>pp. 154-170: lista de razones para fijar el umbral.</t>
         </is>
       </c>
+      <c r="J226" s="7" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n">
@@ -10870,6 +11159,7 @@
           <t>pp. 154-156: «los costes de la condena falsa son relativos al tipo de condena, no a la jurisdicción»; ejemplo del derecho administrativo sancionador.</t>
         </is>
       </c>
+      <c r="J227" s="7" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n">
@@ -10915,6 +11205,7 @@
           <t>p. 164: delitos de corrupción; dificultades probatorias como razón para disminuir la exigencia.</t>
         </is>
       </c>
+      <c r="J228" s="7" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
@@ -10960,6 +11251,7 @@
           <t>p. 166: sin método objetivo para ponderar; riesgo de diseño ineficaz.</t>
         </is>
       </c>
+      <c r="J229" s="7" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n">
@@ -11005,6 +11297,7 @@
           <t>pp. 168-169: desequilibrio de poder entre las partes; redes de corrupción con cargos públicos.</t>
         </is>
       </c>
+      <c r="J230" s="7" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">
@@ -11050,6 +11343,7 @@
           <t>CPEUM art. 41, base VI, incisos a) a d) (inciso d) adicionado DOF 02-06-2026) y LGSMIME art. 78 bis, párr. 2.</t>
         </is>
       </c>
+      <c r="J231" s="7" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n">
@@ -11095,6 +11389,7 @@
           <t>SUP-REC-1388/2018, p. 46: estándar «mínimo» para la determinancia en violencia política.</t>
         </is>
       </c>
+      <c r="J232" s="7" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n">
@@ -11140,6 +11435,7 @@
           <t>pp. 209-210: siete formulaciones de estándares; los tres primeros inspirados en Hempel y Cohen.</t>
         </is>
       </c>
+      <c r="J233" s="7" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n">
@@ -11185,6 +11481,7 @@
           <t>p. 210: estándares 1) a 7).</t>
         </is>
       </c>
+      <c r="J234" s="7" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n">
@@ -11230,6 +11527,7 @@
           <t>p. 215: aun satisfecho el estándar más exigente, «la conclusión es siempre probabilística» (ejemplo del ADN).</t>
         </is>
       </c>
+      <c r="J235" s="7" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n">
@@ -11275,6 +11573,7 @@
           <t>p. 211: adopción del estándar 1) por la jurisprudencia penal portuguesa (nota 10).</t>
         </is>
       </c>
+      <c r="J236" s="7" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n">
@@ -11320,6 +11619,7 @@
           <t>pp. 214-215: transcripción del ADR 3457/2013 (desvirtuar la hipótesis de inocencia alegada; descartar pruebas de descargo).</t>
         </is>
       </c>
+      <c r="J237" s="7" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n">
@@ -11365,6 +11665,7 @@
           <t>Allen en Vázquez (ed.), pp. 55-56: crítica al estándar de Ferrer; la excepción de las hipótesis ad hoc «parece ser ella misma totalmente ad hoc».</t>
         </is>
       </c>
+      <c r="J238" s="7" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n">
@@ -11410,6 +11711,7 @@
           <t>Allen, pp. 56-57: teoría de la plausibilidad relativa; «no es una propuesta normativa sino descriptiva».</t>
         </is>
       </c>
+      <c r="J239" s="7" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n">
@@ -11455,6 +11757,7 @@
           <t>p. 211 (nota 8): tesis de la unidad del razonamiento empírico (González Lagier, Haack).</t>
         </is>
       </c>
+      <c r="J240" s="7" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n">
@@ -11500,6 +11803,7 @@
           <t>Allen, pp. 53-54: el derecho no puede seleccionar sus disputas; variables de un testimonio.</t>
         </is>
       </c>
+      <c r="J241" s="7" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n">
@@ -11545,6 +11849,7 @@
           <t>p. 44: la comprobación del estándar solo en el caso concreto; «la índole de razones» (Dei Vecchi).</t>
         </is>
       </c>
+      <c r="J242" s="7" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n">
@@ -11572,24 +11877,25 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H243" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I243" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 135: los estándares «no describen la realidad, sino un mero desideratum psicológico que no va a ser comprobado».</t>
+        </is>
+      </c>
+      <c r="J243" s="7" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n">
@@ -11617,24 +11923,25 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H244" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H244" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I244" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 136: «sensación absolutamente subjetiva»; lógica aritmética del sistema de valoración legal que sumaba y pesaba pruebas.</t>
+        </is>
+      </c>
+      <c r="J244" s="7" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n">
@@ -11680,6 +11987,7 @@
           <t>Haack, pp. 69-70: la justificación de cargas y estándares «se funda también en consideraciones políticas».</t>
         </is>
       </c>
+      <c r="J245" s="7" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n">
@@ -11725,6 +12033,7 @@
           <t>Art. 16, párrs. 2 y 3, LGSMIME.</t>
         </is>
       </c>
+      <c r="J246" s="7" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n">
@@ -11770,6 +12079,7 @@
           <t>LGSMIME arts. 75.1.k, 77 Ter.2 y 78.1: «plenamente acreditadas» y determinantes.</t>
         </is>
       </c>
+      <c r="J247" s="7" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n">
@@ -11815,6 +12125,7 @@
           <t>Jurisprudencia 44/2024.</t>
         </is>
       </c>
+      <c r="J248" s="7" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n">
@@ -11842,24 +12153,25 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fuera del RIS (PDF en Drive)</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>No figura en el RIS</t>
-        </is>
-      </c>
-      <c r="H249" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
+          <t>carga de la prueba y estandares de prueba. dos reminicencias del pasado_Nieva_Fenanol.pdf (Estudios de Derecho, núm. 170, 2020)</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I249" s="2" t="inlineStr">
         <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
+          <t>p. 130: probatio plena como nivel de convicción máxima; primer intento de estandarización.</t>
+        </is>
+      </c>
+      <c r="J249" s="7" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n">
@@ -11905,6 +12217,7 @@
           <t>Voto razonado, p. 75: «estándar probatorio muy alto, prácticamente imposible de alcanzar».</t>
         </is>
       </c>
+      <c r="J250" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -11918,13 +12231,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="100" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11948,424 +12262,234 @@
           <t>Hallazgo y corrección sugerida</t>
         </is>
       </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Corrección aplicada</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="7" t="n">
         <v>126</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Discrepancia sustantiva</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Sala Superior del Tribunal Electoral del Poder Judicial de la Federación, SUP-REC-1388/2018, sentencia de 30 de septiembre de 2018, p. 48.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>p. 48 existe y expone la regla de la presunción de determinancia (&lt;5 %). Pero la Sala NO la aplicó: la diferencia era de 45,922 votos (11.11 %), por lo que sostuvo que la carga correspondía a quien pretendía la nulidad (pp. 48-49). La tesis afirma que «aplicó la presunción». Sugerencia: «la Sala Superior invocó la presunción de determinancia (&lt;5 %) y, al superar la diferencia ese umbral (11.11 %), atribuyó la carga a quien pedía la nulidad (pp. 48-49)». El argumento de la tesis (confusión carga/estándar) se mantiene.</t>
         </is>
       </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Texto: «aplicó» → «invocó» y se añadió: «Como la diferencia entre el primero y el segundo lugar era de 11.11 por ciento, atribuyó la carga de acreditar la determinancia a quien pretendía la nulidad.» Nota: «p. 48» → «pp. 48 y 49».</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Benfeld, Johann, Los orígenes del concepto de sana crítica, Revista de Estudios Histórico-Jurídicos, Valparaíso, núm. XXXV, 2013, pp. 571 y 572.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>pp. 571-572 respaldan el Reglamento de 1846 (art. 148) y la LEC de 1855 (art. 317). La frase posterior «su propósito fue liberar al juez de ponderar a los testigos en razón de su número» está en p. 577 (y p. 574), no en 571-572. Sugerencia: ampliar a «pp. 571, 572 y 577» o agregar nota a esa frase.</t>
         </is>
       </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «pp. 571 y 572» → «pp. 571, 572 y 577».</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Ibidem, p. 86, nota 35.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>p. 86, nota 35 respalda que no debe haber máximas mejor fundadas que desautoricen el paso. La frase siguiente (desconfiar de reglas construidas ad hoc) está en p. 87, no en p. 86. Sugerencia: «p. 86, nota 35, y p. 87».</t>
         </is>
       </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 86, nota 35» → «p. 86, nota 35, y p. 87».</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Sala Superior del Tribunal Electoral del Poder Judicial de la Federación, SUP-JIN-194/2025 y acumulados, sentencia de 20 de agosto de 2025, magistrado encargado del engrose Felipe Alfredo Fuentes Barrera, párrafos 50 a 60, pp. 11-13.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párrs. 50-60 están en pp. 10-12 (no 11-13). Contenido conforme: requisitos de indicios e inferencias.</t>
         </is>
       </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «pp. 11-13» → «pp. 10-12».</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="7" t="n">
         <v>152</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Ibidem, p. 99.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>La característica «2. Naturaleza objetiva: No debe basarse en percepciones personales del juzgador» está en p. 98, no en p. 99 (p. 99 contiene las características 3 a 5). Sugerencia: «p. 98» o «pp. 98 y 99».</t>
         </is>
       </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 99» → «p. 98».</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="7" t="n">
         <v>156</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Sala Superior del Tribunal Electoral del Poder Judicial de la Federación, SUP-JIN-194/2025 y acumulados, sentencia de 20 de agosto de 2025, párrafo 39, p. 8.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 39 (estándar flexible; imposible demostrar de manera directa) está en p. 7, no en p. 8.</t>
         </is>
       </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 8» → «p. 7».</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="7" t="n">
         <v>157</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Ibidem, párrafo 45, p. 9.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 45 («consecuencia más extrema y lesiva»; plena acreditación) está en p. 8, no en p. 9.</t>
         </is>
       </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 9» → «p. 8».</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="7" t="n">
         <v>158</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Ibidem, párrafo 50, p. 11.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 50 («escuela de libre investigación o libre convencimiento»; «formulación racional y controlable») está en p. 10, no en p. 11.</t>
         </is>
       </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «p. 11» → «p. 10».</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="7" t="n">
         <v>206</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Discrepancia menor</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Ibidem, pp. 78 y 81.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Haack: la metáfora del crucigrama está en p. 78 ✓, pero la afirmación de que una agregación puede avalar la conclusión en grado mayor que sus componentes está en p. 82 (no en p. 81). Sugerencia: «pp. 78 y 82».</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Jordi, Carga de la prueba y estándares de prueba. Dos reminiscencias del pasado, Estudios de Derecho, Medellín, vol. 77, núm. 170, 2020, p. 130.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (Estudios de Derecho, 2020) no figura en el RIS (el RIS registra otra obra del autor: La valoración de la prueba, 2010). No se verificó por instrucción de limitarse al RIS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Carga de la prueba y estándares de prueba, cit., p. 131, nota 56.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Ibidem, p. 132.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Ibidem, p. 133.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>114</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Carga de la prueba y estándares de prueba, cit., p. 118.</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>115</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Ibidem, p. 133.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>116</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Ibidem, p. 134.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, «Carga de la prueba y estándares de prueba...» (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Carga de la prueba y estándares de prueba, cit., p. 128.</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>149</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Carga de la prueba y estándares de prueba, cit., p. 131, nota 54.</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>242</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Jordi, Carga de la prueba y estándares de prueba. Dos reminiscencias del pasado, Estudios de Derecho, Medellín, vol. 77, núm. 170, 2020, p. 135.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>243</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Ibidem, p. 136.</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>248</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Fuera del RIS</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll, Carga de la prueba y estándares de prueba, cit., p. 130.</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Nieva-Fenoll (2020): no figura en el RIS. No verificada.</t>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Nota: «pp. 78 y 81» → «pp. 78 y 82».</t>
         </is>
       </c>
     </row>
@@ -12738,7 +12862,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Obra citada (12 notas en el Cap. I) fuera del RIS.</t>
+          <t>El artículo citado (2020) no está en el RIS pero sí en el Drive; las 12 notas se verificaron y son conformes. Conviene agregarlo al RIS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revierte correcciones de las notas 60 y 156-158 y agrega RIS corregido
La paginación del SUP-JIN-194/2025 va al pie de página; las páginas que
cita la tesis son correctas. Se revierten esas cuatro correcciones en
ambos .docx y se actualiza el informe del Capítulo I (fe de erratas).
Se añade fuentes_tesis-v3.ris con los datos bibliográficos corregidos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFqB7qFXyXBvPWdV8axcUP
</commit_message>
<xml_diff>
--- a/Verificacion_citas_Cap_I.xlsx
+++ b/Verificacion_citas_Cap_I.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -638,10 +638,11 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(1) Ferrer, Prueba sin convicción: el tramo impreso pp. 139-148 no está paginado en las copias descargables; la nota 123 se localizó por contenido (±1 página). (2) Laudan, Truth…, Devis Echandía y SUP-JIN-194/2025 se leyeron mediante el texto que extrae Drive, por exceder el límite de descarga de 10 MB.</t>
-        </is>
-      </c>
-    </row>
+          <t>(1) Ferrer, Prueba sin convicción: el tramo impreso pp. 139-148 no está paginado en las copias descargables; la nota 123 se localizó por contenido (±1 página). (2) Laudan, Truth…, Devis Echandía y SUP-JIN-194/2025 se leyeron mediante el texto que extrae Drive, por exceder el límite de descarga de 10 MB. (3) En SUP-JIN-194/2025 el número de página figura al pie; la localización se contrastó con el PDF original.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
@@ -650,7 +651,19 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Las 9 discrepancias se subsanaron en «Tesis_Cap_I-V_citas_corregidas.docx» con control de cambios (autor: Claude, verificación de citas). Se entrega también una versión limpia con los cambios aceptados.</t>
+          <t>Las 5 discrepancias se subsanaron en «Tesis_Cap_I-V_citas_corregidas.docx» con control de cambios (autor: Claude, verificación de citas). Se entrega también una versión limpia con los cambios aceptados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fe de erratas (26-09-2026)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>En la primera entrega se clasificaron como «discrepancia menor» las notas 60, 156, 157 y 158 (SUP-JIN-194/2025) por un supuesto desfase de una página. Al cotejar el PDF original se comprobó que el número de página va al pie y que las páginas citadas en la tesis son correctas. Esas cuatro correcciones se revirtieron en ambos .docx.</t>
         </is>
       </c>
     </row>
@@ -3489,19 +3502,19 @@
           <t>SUP-JIN-194-2025… compressed-1-300 (texto extraído por Drive)</t>
         </is>
       </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párrs. 50-60 están en pp. 10-12 (no 11-13). Contenido conforme: requisitos de indicios e inferencias.</t>
+          <t>SUP-JIN-194/2025, párrs. 50-60, pp. 11-13 (paginación al pie de página): requisitos de indicios e inferencias; contenido conforme.</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>Nota: «pp. 11-13» → «pp. 10-12».</t>
+          <t>Ninguna. La corrección inicial se revirtió: el número de página del SUP-JIN-194/2025 va al pie, no en el encabezado, y la cita de la tesis es exacta.</t>
         </is>
       </c>
     </row>
@@ -7917,19 +7930,19 @@
           <t>SUP-JIN-194-2025… compressed-1-300 (texto extraído por Drive)</t>
         </is>
       </c>
-      <c r="H157" s="4" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 39 (estándar flexible; imposible demostrar de manera directa) está en p. 7, no en p. 8.</t>
+          <t>SUP-JIN-194/2025, párr. 39, p. 8: estándar flexible; imposibilidad de demostración directa.</t>
         </is>
       </c>
       <c r="J157" s="7" t="inlineStr">
         <is>
-          <t>Nota: «p. 8» → «p. 7».</t>
+          <t>Ninguna. La corrección inicial se revirtió: el número de página del SUP-JIN-194/2025 va al pie, no en el encabezado, y la cita de la tesis es exacta.</t>
         </is>
       </c>
     </row>
@@ -7967,19 +7980,19 @@
           <t>SUP-JIN-194-2025… compressed-1-300 (texto extraído por Drive)</t>
         </is>
       </c>
-      <c r="H158" s="4" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 45 («consecuencia más extrema y lesiva»; plena acreditación) está en p. 8, no en p. 9.</t>
+          <t>SUP-JIN-194/2025, párr. 45, p. 9: nulidad como «consecuencia más extrema y lesiva»; plena acreditación.</t>
         </is>
       </c>
       <c r="J158" s="7" t="inlineStr">
         <is>
-          <t>Nota: «p. 9» → «p. 8».</t>
+          <t>Ninguna. La corrección inicial se revirtió: el número de página del SUP-JIN-194/2025 va al pie, no en el encabezado, y la cita de la tesis es exacta.</t>
         </is>
       </c>
     </row>
@@ -8017,19 +8030,19 @@
           <t>SUP-JIN-194-2025… compressed-1-300 (texto extraído por Drive)</t>
         </is>
       </c>
-      <c r="H159" s="4" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 50 («escuela de libre investigación o libre convencimiento»; «formulación racional y controlable») está en p. 10, no en p. 11.</t>
+          <t>SUP-JIN-194/2025, párr. 50, p. 11: «escuela de libre investigación o libre convencimiento»; formulación racional y controlable.</t>
         </is>
       </c>
       <c r="J159" s="7" t="inlineStr">
         <is>
-          <t>Nota: «p. 11» → «p. 10».</t>
+          <t>Ninguna. La corrección inicial se revirtió: el número de página del SUP-JIN-194/2025 va al pie, no en el encabezado, y la cita de la tesis es exacta.</t>
         </is>
       </c>
     </row>
@@ -12231,7 +12244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12345,7 +12358,7 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
-        <v>60</v>
+        <v>152</v>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
@@ -12354,23 +12367,23 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Sala Superior del Tribunal Electoral del Poder Judicial de la Federación, SUP-JIN-194/2025 y acumulados, sentencia de 20 de agosto de 2025, magistrado encargado del engrose Felipe Alfredo Fuentes Barrera, párrafos 50 a 60, pp. 11-13.</t>
+          <t>Ibidem, p. 99.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párrs. 50-60 están en pp. 10-12 (no 11-13). Contenido conforme: requisitos de indicios e inferencias.</t>
+          <t>La característica «2. Naturaleza objetiva: No debe basarse en percepciones personales del juzgador» está en p. 98, no en p. 99 (p. 99 contiene las características 3 a 5). Sugerencia: «p. 98» o «pp. 98 y 99».</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Nota: «pp. 11-13» → «pp. 10-12».</t>
+          <t>Nota: «p. 99» → «p. 98».</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>152</v>
+        <v>206</v>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
@@ -12379,115 +12392,15 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Ibidem, p. 99.</t>
+          <t>Ibidem, pp. 78 y 81.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>La característica «2. Naturaleza objetiva: No debe basarse en percepciones personales del juzgador» está en p. 98, no en p. 99 (p. 99 contiene las características 3 a 5). Sugerencia: «p. 98» o «pp. 98 y 99».</t>
+          <t>Haack: la metáfora del crucigrama está en p. 78 ✓, pero la afirmación de que una agregación puede avalar la conclusión en grado mayor que sus componentes está en p. 82 (no en p. 81). Sugerencia: «pp. 78 y 82».</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Nota: «p. 99» → «p. 98».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
-        <v>156</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Sala Superior del Tribunal Electoral del Poder Judicial de la Federación, SUP-JIN-194/2025 y acumulados, sentencia de 20 de agosto de 2025, párrafo 39, p. 8.</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 39 (estándar flexible; imposible demostrar de manera directa) está en p. 7, no en p. 8.</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Nota: «p. 8» → «p. 7».</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>157</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Ibidem, párrafo 45, p. 9.</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 45 («consecuencia más extrema y lesiva»; plena acreditación) está en p. 8, no en p. 9.</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Nota: «p. 9» → «p. 8».</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
-        <v>158</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Ibidem, párrafo 50, p. 11.</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Patrón en SUP-JIN-194/2025: los párrafos citados son correctos, pero la numeración impresa de la sentencia sitúa cada párrafo una página antes de la que indica la tesis (probable uso del número del visor PDF). Párr. 50 («escuela de libre investigación o libre convencimiento»; «formulación racional y controlable») está en p. 10, no en p. 11.</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Nota: «p. 11» → «p. 10».</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>206</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Discrepancia menor</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Ibidem, pp. 78 y 81.</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Haack: la metáfora del crucigrama está en p. 78 ✓, pero la afirmación de que una agregación puede avalar la conclusión en grado mayor que sus componentes está en p. 82 (no en p. 81). Sugerencia: «pp. 78 y 82».</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Nota: «pp. 78 y 81» → «pp. 78 y 82».</t>
         </is>

</xml_diff>